<commit_message>
Add comprehensive tests for PL/SQL DDL, semantics, and program model validation
- Introduced tests for rendering PL/SQL program DDL and assertions in `plsql-ddl.test.ts`.
- Added extensive validation tests for PL/SQL source inspection and lexing in `plsql.test.ts`.
- Implemented tests for program model selection and policy schemas in `program-model.test.ts`.
- Created tests for program semantics, including validation, SQL generation, and dependency management in `program-semantics.test.ts`.
- Ensured coverage for edge cases, such as recursive dependencies, cross-owner access, and automatic grants.
</commit_message>
<xml_diff>
--- a/examples/data-dictionary.xlsx
+++ b/examples/data-dictionary.xlsx
@@ -11,15 +11,17 @@
     <sheet sheetId="5" name="Indexes" state="visible" r:id="rId8"/>
     <sheet sheetId="6" name="Views" state="visible" r:id="rId9"/>
     <sheet sheetId="7" name="View Dependencies" state="visible" r:id="rId10"/>
-    <sheet sheetId="8" name="Prerequisites" state="visible" r:id="rId11"/>
-    <sheet sheetId="9" name="Diagnostics" state="visible" r:id="rId12"/>
+    <sheet sheetId="8" name="Programs" state="visible" r:id="rId11"/>
+    <sheet sheetId="9" name="Program Dependencies" state="visible" r:id="rId12"/>
+    <sheet sheetId="10" name="Prerequisites" state="visible" r:id="rId13"/>
+    <sheet sheetId="11" name="Diagnostics" state="visible" r:id="rId14"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="142">
   <si>
     <t>Property</t>
   </si>
@@ -66,6 +68,18 @@
     <t>Target view count</t>
   </si>
   <si>
+    <t>Selection version</t>
+  </si>
+  <si>
+    <t>Target procedure count</t>
+  </si>
+  <si>
+    <t>Target package count</t>
+  </si>
+  <si>
+    <t>Included program count</t>
+  </si>
+  <si>
     <t>Included table count</t>
   </si>
   <si>
@@ -393,16 +407,34 @@
     <t>Database Link</t>
   </si>
   <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>AUTHID</t>
+  </si>
+  <si>
+    <t>Unit</t>
+  </si>
+  <si>
+    <t>Editionable</t>
+  </si>
+  <si>
+    <t>Body Required</t>
+  </si>
+  <si>
+    <t>Referenced Owner</t>
+  </si>
+  <si>
+    <t>Referenced Name</t>
+  </si>
+  <si>
+    <t>Oracle Maintained</t>
+  </si>
+  <si>
     <t>Required By Owner</t>
   </si>
   <si>
     <t>Required By Name</t>
-  </si>
-  <si>
-    <t>Referenced Owner</t>
-  </si>
-  <si>
-    <t>Referenced Name</t>
   </si>
   <si>
     <t>Severity</t>
@@ -818,7 +850,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -845,7 +877,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="2">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -928,8 +960,109 @@
         <v>0</v>
       </c>
     </row>
+    <row r="14" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17" s="2">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:B1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="19" customWidth="1"/>
+    <col min="2" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="17" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="6" max="6" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="48" style="4" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>141</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -952,57 +1085,57 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="H2" s="3">
         <v>2</v>
@@ -1016,23 +1149,23 @@
     </row>
     <row r="3" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="H3" s="2">
         <v>2</v>
@@ -1075,91 +1208,91 @@
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="T1" s="5" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="D2" s="3">
         <v>1</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="G2" s="2"/>
       <c r="H2" s="3" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="I2" s="3">
         <v>22</v>
@@ -1175,17 +1308,17 @@
         <v>0</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="O2" s="2"/>
       <c r="P2" s="3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="S2" s="2"/>
       <c r="T2" s="2"/>
@@ -1193,24 +1326,24 @@
     </row>
     <row r="3" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="D3" s="2">
         <v>2</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
       <c r="H3" s="2" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="I3" s="2">
         <v>22</v>
@@ -1226,17 +1359,17 @@
         <v>0</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="O3" s="2"/>
       <c r="P3" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="S3" s="2"/>
       <c r="T3" s="2"/>
@@ -1244,24 +1377,24 @@
     </row>
     <row r="4" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D4" s="3">
         <v>1</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
       <c r="H4" s="3" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="I4" s="3">
         <v>22</v>
@@ -1277,17 +1410,17 @@
         <v>0</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="O4" s="2"/>
       <c r="P4" s="3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="Q4" s="3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="R4" s="3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="S4" s="2"/>
       <c r="T4" s="2"/>
@@ -1295,24 +1428,24 @@
     </row>
     <row r="5" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D5" s="2">
         <v>2</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
       <c r="H5" s="2" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="I5" s="2">
         <v>22</v>
@@ -1328,17 +1461,17 @@
         <v>0</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="O5" s="2"/>
       <c r="P5" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="Q5" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="R5" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="S5" s="2"/>
       <c r="T5" s="2"/>
@@ -1377,199 +1510,199 @@
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="2" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="F2" s="3">
         <v>1</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="L2" s="2"/>
       <c r="M2" s="3" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="N2" s="2"/>
       <c r="O2" s="2"/>
       <c r="P2" s="3" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="F3" s="2">
         <v>2</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="L3" s="2"/>
       <c r="M3" s="2" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="N3" s="2"/>
       <c r="O3" s="2"/>
       <c r="P3" s="2" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="S3" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="T3" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="F4" s="3">
         <v>1</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
@@ -1578,48 +1711,48 @@
       <c r="L4" s="2"/>
       <c r="M4" s="2"/>
       <c r="N4" s="3" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="P4" s="3" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="Q4" s="3" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="R4" s="3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="S4" s="3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="T4" s="3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="F5" s="2">
         <v>2</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
@@ -1628,160 +1761,160 @@
       <c r="L5" s="2"/>
       <c r="M5" s="2"/>
       <c r="N5" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="P5" s="2" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="Q5" s="2" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="R5" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="S5" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="T5" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
     </row>
     <row r="6" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="F6" s="3">
         <v>1</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="L6" s="2"/>
       <c r="M6" s="3" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="N6" s="2"/>
       <c r="O6" s="2"/>
       <c r="P6" s="3" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="Q6" s="3" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="R6" s="3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="S6" s="3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="T6" s="3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
     </row>
     <row r="7" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="F7" s="2">
         <v>2</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="L7" s="2"/>
       <c r="M7" s="2" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
       <c r="P7" s="2" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="Q7" s="2" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="R7" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="S7" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="T7" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
     </row>
     <row r="8" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="F8" s="3">
         <v>1</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
@@ -1790,48 +1923,48 @@
       <c r="L8" s="2"/>
       <c r="M8" s="2"/>
       <c r="N8" s="3" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="O8" s="3" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="P8" s="3" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="Q8" s="3" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="R8" s="3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="S8" s="3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="T8" s="3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
     </row>
     <row r="9" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="F9" s="2">
         <v>2</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
@@ -1840,25 +1973,25 @@
       <c r="L9" s="2"/>
       <c r="M9" s="2"/>
       <c r="N9" s="2" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="P9" s="2" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="Q9" s="2" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="R9" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="S9" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="T9" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -1886,214 +2019,214 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
     </row>
     <row r="2" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="K2" s="3">
         <v>1</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="M2" s="2"/>
       <c r="N2" s="3" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="3" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="K3" s="2">
         <v>2</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="M3" s="2"/>
       <c r="N3" s="2" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="K4" s="3">
         <v>1</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="M4" s="2"/>
       <c r="N4" s="3" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="5" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="K5" s="2">
         <v>2</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="M5" s="2"/>
       <c r="N5" s="2" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>
@@ -2119,49 +2252,49 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -2185,28 +2318,28 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
   </sheetData>
@@ -2218,38 +2351,45 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="19" customWidth="1"/>
-    <col min="2" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="17" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="15" customWidth="1"/>
+    <col min="1" max="7" width="12" customWidth="1"/>
+    <col min="8" max="8" width="13" customWidth="1"/>
+    <col min="9" max="9" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>124</v>
+        <v>23</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>126</v>
+        <v>69</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>127</v>
+        <v>25</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>94</v>
+        <v>129</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>123</v>
+        <v>130</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>132</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F1"/>
+  <autoFilter ref="A1:I1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -2257,29 +2397,45 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="48" style="4" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="17" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+    <col min="8" max="8" width="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>128</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>129</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="D1" s="5" t="s">
-        <v>131</v>
+      <c r="D1" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>135</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D1"/>
+  <autoFilter ref="A1:H1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Add comprehensive tests for object grants, operation order, program DDL, sequences, and synonyms
- Introduced tests for explicit grants to validate rejection of unrelated owners, wrong types, synonyms, self-grants, and unsupported privileges.
- Added tests to ensure correct operation order for functions, sequences, and package bodies, preventing false cycles.
- Implemented tests for CLOB transport and program wrapper to verify accurate DDL generation and resource management.
- Created tests for sequence behavior, including bounds, increments, and cache combinations, ensuring proper validation.
- Developed tests for synonyms to check dependency resolution, alias chains, and external alias links, ensuring correct SQL generation.
</commit_message>
<xml_diff>
--- a/examples/data-dictionary.xlsx
+++ b/examples/data-dictionary.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="140">
   <si>
     <t>Property</t>
   </si>
@@ -64,6 +64,30 @@
   </si>
   <si>
     <t>Target view count</t>
+  </si>
+  <si>
+    <t>Target procedure count</t>
+  </si>
+  <si>
+    <t>Target function count</t>
+  </si>
+  <si>
+    <t>Target package count</t>
+  </si>
+  <si>
+    <t>Program unit count</t>
+  </si>
+  <si>
+    <t>Sequence count</t>
+  </si>
+  <si>
+    <t>Synonym count</t>
+  </si>
+  <si>
+    <t>Program definitions</t>
+  </si>
+  <si>
+    <t>Exact source and dependency metadata are authoritative in JSON.</t>
   </si>
   <si>
     <t>Included table count</t>
@@ -818,7 +842,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -845,7 +869,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="2">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -901,7 +925,7 @@
         <v>15</v>
       </c>
       <c r="B10" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -925,6 +949,62 @@
         <v>18</v>
       </c>
       <c r="B13" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B17" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B18" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B19" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" s="3">
         <v>0</v>
       </c>
     </row>
@@ -952,57 +1032,57 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="H2" s="3">
         <v>2</v>
@@ -1016,23 +1096,23 @@
     </row>
     <row r="3" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="H3" s="2">
         <v>2</v>
@@ -1075,91 +1155,91 @@
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="T1" s="5" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="D2" s="3">
         <v>1</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="G2" s="2"/>
       <c r="H2" s="3" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="I2" s="3">
         <v>22</v>
@@ -1175,17 +1255,17 @@
         <v>0</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="O2" s="2"/>
       <c r="P2" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="S2" s="2"/>
       <c r="T2" s="2"/>
@@ -1193,24 +1273,24 @@
     </row>
     <row r="3" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="D3" s="2">
         <v>2</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
       <c r="H3" s="2" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="I3" s="2">
         <v>22</v>
@@ -1226,17 +1306,17 @@
         <v>0</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="O3" s="2"/>
       <c r="P3" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="S3" s="2"/>
       <c r="T3" s="2"/>
@@ -1244,24 +1324,24 @@
     </row>
     <row r="4" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="D4" s="3">
         <v>1</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
       <c r="H4" s="3" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="I4" s="3">
         <v>22</v>
@@ -1277,17 +1357,17 @@
         <v>0</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="O4" s="2"/>
       <c r="P4" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="Q4" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="R4" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="S4" s="2"/>
       <c r="T4" s="2"/>
@@ -1295,24 +1375,24 @@
     </row>
     <row r="5" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="D5" s="2">
         <v>2</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
       <c r="H5" s="2" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="I5" s="2">
         <v>22</v>
@@ -1328,17 +1408,17 @@
         <v>0</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="O5" s="2"/>
       <c r="P5" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="Q5" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="R5" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="S5" s="2"/>
       <c r="T5" s="2"/>
@@ -1377,199 +1457,199 @@
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="F2" s="3">
         <v>1</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="L2" s="2"/>
       <c r="M2" s="3" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="N2" s="2"/>
       <c r="O2" s="2"/>
       <c r="P2" s="3" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="F3" s="2">
         <v>2</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="L3" s="2"/>
       <c r="M3" s="2" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="N3" s="2"/>
       <c r="O3" s="2"/>
       <c r="P3" s="2" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="S3" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="T3" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="F4" s="3">
         <v>1</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
@@ -1578,48 +1658,48 @@
       <c r="L4" s="2"/>
       <c r="M4" s="2"/>
       <c r="N4" s="3" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="P4" s="3" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="Q4" s="3" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="R4" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="S4" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="T4" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="F5" s="2">
         <v>2</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
@@ -1628,160 +1708,160 @@
       <c r="L5" s="2"/>
       <c r="M5" s="2"/>
       <c r="N5" s="2" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="P5" s="2" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="Q5" s="2" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="R5" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="S5" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="T5" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="F6" s="3">
         <v>1</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="L6" s="2"/>
       <c r="M6" s="3" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="N6" s="2"/>
       <c r="O6" s="2"/>
       <c r="P6" s="3" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="Q6" s="3" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="R6" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="S6" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="T6" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
     </row>
     <row r="7" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="F7" s="2">
         <v>2</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="L7" s="2"/>
       <c r="M7" s="2" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
       <c r="P7" s="2" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="Q7" s="2" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="R7" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="S7" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="T7" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="F8" s="3">
         <v>1</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
@@ -1790,48 +1870,48 @@
       <c r="L8" s="2"/>
       <c r="M8" s="2"/>
       <c r="N8" s="3" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="O8" s="3" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="P8" s="3" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="Q8" s="3" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="R8" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="S8" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="T8" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="F9" s="2">
         <v>2</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
@@ -1840,25 +1920,25 @@
       <c r="L9" s="2"/>
       <c r="M9" s="2"/>
       <c r="N9" s="2" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="P9" s="2" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="Q9" s="2" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="R9" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="S9" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="T9" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -1886,214 +1966,214 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="K2" s="3">
         <v>1</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="M2" s="2"/>
       <c r="N2" s="3" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="K3" s="2">
         <v>2</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="M3" s="2"/>
       <c r="N3" s="2" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
     </row>
     <row r="4" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="K4" s="3">
         <v>1</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="M4" s="2"/>
       <c r="N4" s="3" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="K5" s="2">
         <v>2</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="M5" s="2"/>
       <c r="N5" s="2" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -2119,49 +2199,49 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -2185,28 +2265,28 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
     </row>
   </sheetData>
@@ -2230,22 +2310,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
     </row>
   </sheetData>
@@ -2266,16 +2346,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add comprehensive tests for catalog programs and sequences
- Introduced unit tests for OracleCatalog's program and sequence functionalities, ensuring proper handling of metadata, visibility, and error cases.
- Implemented integration tests to validate program metadata extraction, privileges, and sequence resets in an Oracle environment.
- Enhanced test coverage for edge cases, including handling of CLOBs, program dependencies, and sequence configurations.
- Validated SQL generation and execution order for various database objects, ensuring compliance with Oracle's constraints and behaviors.
</commit_message>
<xml_diff>
--- a/examples/data-dictionary.xlsx
+++ b/examples/data-dictionary.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="140">
   <si>
     <t>Property</t>
   </si>
@@ -66,10 +66,34 @@
     <t>Target view count</t>
   </si>
   <si>
+    <t>Target package count</t>
+  </si>
+  <si>
+    <t>Target procedure count</t>
+  </si>
+  <si>
+    <t>Target function count</t>
+  </si>
+  <si>
+    <t>Target sequence count</t>
+  </si>
+  <si>
     <t>Included table count</t>
   </si>
   <si>
     <t>Included view count</t>
+  </si>
+  <si>
+    <t>Included program count</t>
+  </si>
+  <si>
+    <t>Included sequence count</t>
+  </si>
+  <si>
+    <t>Dictionary scope</t>
+  </si>
+  <si>
+    <t>Tables and views; program DDL is not included.</t>
   </si>
   <si>
     <t>Prerequisite count</t>
@@ -818,7 +842,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -845,7 +869,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="2">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -901,7 +925,7 @@
         <v>15</v>
       </c>
       <c r="B10" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -925,6 +949,62 @@
         <v>18</v>
       </c>
       <c r="B13" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B19" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" s="3">
         <v>0</v>
       </c>
     </row>
@@ -952,57 +1032,57 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="H2" s="3">
         <v>2</v>
@@ -1016,23 +1096,23 @@
     </row>
     <row r="3" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="H3" s="2">
         <v>2</v>
@@ -1075,91 +1155,91 @@
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="T1" s="5" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="D2" s="3">
         <v>1</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="G2" s="2"/>
       <c r="H2" s="3" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="I2" s="3">
         <v>22</v>
@@ -1175,17 +1255,17 @@
         <v>0</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="O2" s="2"/>
       <c r="P2" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="S2" s="2"/>
       <c r="T2" s="2"/>
@@ -1193,24 +1273,24 @@
     </row>
     <row r="3" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="D3" s="2">
         <v>2</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
       <c r="H3" s="2" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="I3" s="2">
         <v>22</v>
@@ -1226,17 +1306,17 @@
         <v>0</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="O3" s="2"/>
       <c r="P3" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="S3" s="2"/>
       <c r="T3" s="2"/>
@@ -1244,24 +1324,24 @@
     </row>
     <row r="4" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="D4" s="3">
         <v>1</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
       <c r="H4" s="3" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="I4" s="3">
         <v>22</v>
@@ -1277,17 +1357,17 @@
         <v>0</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="O4" s="2"/>
       <c r="P4" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="Q4" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="R4" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="S4" s="2"/>
       <c r="T4" s="2"/>
@@ -1295,24 +1375,24 @@
     </row>
     <row r="5" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="D5" s="2">
         <v>2</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
       <c r="H5" s="2" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="I5" s="2">
         <v>22</v>
@@ -1328,17 +1408,17 @@
         <v>0</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="O5" s="2"/>
       <c r="P5" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="Q5" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="R5" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="S5" s="2"/>
       <c r="T5" s="2"/>
@@ -1377,199 +1457,199 @@
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="F2" s="3">
         <v>1</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="L2" s="2"/>
       <c r="M2" s="3" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="N2" s="2"/>
       <c r="O2" s="2"/>
       <c r="P2" s="3" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="F3" s="2">
         <v>2</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="L3" s="2"/>
       <c r="M3" s="2" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="N3" s="2"/>
       <c r="O3" s="2"/>
       <c r="P3" s="2" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="S3" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="T3" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="F4" s="3">
         <v>1</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
@@ -1578,48 +1658,48 @@
       <c r="L4" s="2"/>
       <c r="M4" s="2"/>
       <c r="N4" s="3" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="P4" s="3" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="Q4" s="3" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="R4" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="S4" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="T4" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="F5" s="2">
         <v>2</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
@@ -1628,160 +1708,160 @@
       <c r="L5" s="2"/>
       <c r="M5" s="2"/>
       <c r="N5" s="2" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="P5" s="2" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="Q5" s="2" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="R5" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="S5" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="T5" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="F6" s="3">
         <v>1</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="L6" s="2"/>
       <c r="M6" s="3" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="N6" s="2"/>
       <c r="O6" s="2"/>
       <c r="P6" s="3" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="Q6" s="3" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="R6" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="S6" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="T6" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
     </row>
     <row r="7" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="F7" s="2">
         <v>2</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="L7" s="2"/>
       <c r="M7" s="2" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
       <c r="P7" s="2" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="Q7" s="2" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="R7" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="S7" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="T7" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="F8" s="3">
         <v>1</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
@@ -1790,48 +1870,48 @@
       <c r="L8" s="2"/>
       <c r="M8" s="2"/>
       <c r="N8" s="3" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="O8" s="3" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="P8" s="3" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="Q8" s="3" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="R8" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="S8" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="T8" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="F9" s="2">
         <v>2</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
@@ -1840,25 +1920,25 @@
       <c r="L9" s="2"/>
       <c r="M9" s="2"/>
       <c r="N9" s="2" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="P9" s="2" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="Q9" s="2" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="R9" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="S9" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="T9" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -1886,214 +1966,214 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="K2" s="3">
         <v>1</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="M2" s="2"/>
       <c r="N2" s="3" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="K3" s="2">
         <v>2</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="M3" s="2"/>
       <c r="N3" s="2" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
     </row>
     <row r="4" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="K4" s="3">
         <v>1</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="M4" s="2"/>
       <c r="N4" s="3" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="K5" s="2">
         <v>2</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="M5" s="2"/>
       <c r="N5" s="2" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -2119,49 +2199,49 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -2185,28 +2265,28 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
     </row>
   </sheetData>
@@ -2230,22 +2310,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
     </row>
   </sheetData>
@@ -2266,16 +2346,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add synonym management functionality
- Introduced a new JSON schema for synonyms in `examples/synonyms.objects.json`.
- Implemented synonym reading and resolution logic in `src/catalog-synonyms.ts`.
- Created rendering and validation functions for synonyms in `src/synonyms.ts`.
- Added unit tests for synonym catalog functionality in `test/catalog-synonyms.test.ts`.
- Developed integration tests for synonym handling in `test/integration/synonyms.test.ts`.
- Implemented comprehensive tests for synonym extraction and validation in `test/synonyms.test.ts`.
</commit_message>
<xml_diff>
--- a/examples/data-dictionary.xlsx
+++ b/examples/data-dictionary.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="142">
   <si>
     <t>Property</t>
   </si>
@@ -73,6 +73,12 @@
   </si>
   <si>
     <t>Target function count</t>
+  </si>
+  <si>
+    <t>Target synonym count</t>
+  </si>
+  <si>
+    <t>Included synonym count</t>
   </si>
   <si>
     <t>Target sequence count</t>
@@ -842,7 +848,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -869,7 +875,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="2">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -957,7 +963,7 @@
         <v>19</v>
       </c>
       <c r="B14" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -973,7 +979,7 @@
         <v>21</v>
       </c>
       <c r="B16" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -988,13 +994,13 @@
       <c r="A18" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B18" s="3" t="s">
-        <v>24</v>
+      <c r="B18" s="3">
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B19" s="2">
         <v>0</v>
@@ -1002,9 +1008,25 @@
     </row>
     <row r="20" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B20" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B20" s="3">
+    </row>
+    <row r="21" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B21" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B22" s="3">
         <v>0</v>
       </c>
     </row>
@@ -1032,57 +1054,57 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H2" s="3">
         <v>2</v>
@@ -1096,23 +1118,23 @@
     </row>
     <row r="3" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H3" s="2">
         <v>2</v>
@@ -1155,91 +1177,91 @@
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="T1" s="5" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D2" s="3">
         <v>1</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="G2" s="2"/>
       <c r="H2" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I2" s="3">
         <v>22</v>
@@ -1255,17 +1277,17 @@
         <v>0</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="O2" s="2"/>
       <c r="P2" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="S2" s="2"/>
       <c r="T2" s="2"/>
@@ -1273,24 +1295,24 @@
     </row>
     <row r="3" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D3" s="2">
         <v>2</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
       <c r="H3" s="2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I3" s="2">
         <v>22</v>
@@ -1306,17 +1328,17 @@
         <v>0</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="O3" s="2"/>
       <c r="P3" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="S3" s="2"/>
       <c r="T3" s="2"/>
@@ -1324,24 +1346,24 @@
     </row>
     <row r="4" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D4" s="3">
         <v>1</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
       <c r="H4" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I4" s="3">
         <v>22</v>
@@ -1357,17 +1379,17 @@
         <v>0</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="O4" s="2"/>
       <c r="P4" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="Q4" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="R4" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="S4" s="2"/>
       <c r="T4" s="2"/>
@@ -1375,24 +1397,24 @@
     </row>
     <row r="5" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D5" s="2">
         <v>2</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
       <c r="H5" s="2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I5" s="2">
         <v>22</v>
@@ -1408,17 +1430,17 @@
         <v>0</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="O5" s="2"/>
       <c r="P5" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="Q5" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="R5" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="S5" s="2"/>
       <c r="T5" s="2"/>
@@ -1457,199 +1479,199 @@
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F2" s="3">
         <v>1</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="L2" s="2"/>
       <c r="M2" s="3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="N2" s="2"/>
       <c r="O2" s="2"/>
       <c r="P2" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F3" s="2">
         <v>2</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="L3" s="2"/>
       <c r="M3" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="N3" s="2"/>
       <c r="O3" s="2"/>
       <c r="P3" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="S3" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="T3" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F4" s="3">
         <v>1</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
@@ -1658,48 +1680,48 @@
       <c r="L4" s="2"/>
       <c r="M4" s="2"/>
       <c r="N4" s="3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="P4" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="Q4" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="R4" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="S4" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="T4" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F5" s="2">
         <v>2</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
@@ -1708,160 +1730,160 @@
       <c r="L5" s="2"/>
       <c r="M5" s="2"/>
       <c r="N5" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="P5" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="Q5" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="R5" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="S5" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="T5" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="6" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F6" s="3">
         <v>1</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="L6" s="2"/>
       <c r="M6" s="3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="N6" s="2"/>
       <c r="O6" s="2"/>
       <c r="P6" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="Q6" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="R6" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="S6" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="T6" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="7" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F7" s="2">
         <v>2</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="L7" s="2"/>
       <c r="M7" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
       <c r="P7" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="Q7" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="R7" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="S7" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="T7" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="8" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F8" s="3">
         <v>1</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
@@ -1870,48 +1892,48 @@
       <c r="L8" s="2"/>
       <c r="M8" s="2"/>
       <c r="N8" s="3" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O8" s="3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P8" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="Q8" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="R8" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="S8" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="T8" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="9" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F9" s="2">
         <v>2</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
@@ -1920,25 +1942,25 @@
       <c r="L9" s="2"/>
       <c r="M9" s="2"/>
       <c r="N9" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P9" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="Q9" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="R9" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="S9" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="T9" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -1966,214 +1988,214 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="K2" s="3">
         <v>1</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="M2" s="2"/>
       <c r="N2" s="3" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="3" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="K3" s="2">
         <v>2</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="M3" s="2"/>
       <c r="N3" s="2" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="J4" s="3" t="s">
         <v>44</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>42</v>
       </c>
       <c r="K4" s="3">
         <v>1</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="M4" s="2"/>
       <c r="N4" s="3" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="5" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="J5" s="2" t="s">
         <v>44</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>42</v>
       </c>
       <c r="K5" s="2">
         <v>2</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="M5" s="2"/>
       <c r="N5" s="2" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -2199,49 +2221,49 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -2265,28 +2287,28 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
   </sheetData>
@@ -2310,22 +2332,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>133</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>131</v>
       </c>
     </row>
   </sheetData>
@@ -2346,16 +2368,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: implement explicit table selection and FK omission in extraction
- Introduced a new artifact format version (6) that enforces explicit table selection.
- Removed automatic inclusion of foreign keys and view dependencies that are not explicitly selected.
- Updated source and target schemas to reject older versions (1-5) and enforce the new contract.
- Added diagnostics for omitted foreign keys and unselected view tables.
- Enhanced tests to cover new selection behavior, including independent assertions for partial selections.
- Documented changes in ADR 0009 and updated feature documentation to reflect the new extraction rules.
</commit_message>
<xml_diff>
--- a/examples/data-dictionary.xlsx
+++ b/examples/data-dictionary.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="125">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Extraction timestamp</t>
   </si>
   <si>
-    <t>2026-09-22T00:00:00.000Z</t>
+    <t>2026-10-01T12:00:00.000Z</t>
   </si>
   <si>
     <t>Target table count</t>
@@ -129,15 +129,6 @@
     <t/>
   </si>
   <si>
-    <t>SHARED</t>
-  </si>
-  <si>
-    <t>PARENT</t>
-  </si>
-  <si>
-    <t>direct-parent</t>
-  </si>
-  <si>
     <t>Table Owner</t>
   </si>
   <si>
@@ -264,39 +255,15 @@
     <t>Rely</t>
   </si>
   <si>
-    <t>FK_CHILD_PARENT</t>
-  </si>
-  <si>
-    <t>foreign-key</t>
-  </si>
-  <si>
-    <t>PK_PARENT</t>
-  </si>
-  <si>
-    <t>NO ACTION</t>
+    <t>PK_CHILD</t>
+  </si>
+  <si>
+    <t>primary-key</t>
   </si>
   <si>
     <t>TRUE</t>
   </si>
   <si>
-    <t>PK_CHILD</t>
-  </si>
-  <si>
-    <t>primary-key</t>
-  </si>
-  <si>
-    <t>FK_PARENT_GRANDPARENT</t>
-  </si>
-  <si>
-    <t>OTHER</t>
-  </si>
-  <si>
-    <t>GRANDPARENT</t>
-  </si>
-  <si>
-    <t>PK_GRANDPARENT</t>
-  </si>
-  <si>
     <t>Index Owner</t>
   </si>
   <si>
@@ -415,6 +382,18 @@
   </si>
   <si>
     <t>Message</t>
+  </si>
+  <si>
+    <t>change</t>
+  </si>
+  <si>
+    <t>OMIT_UNSELECTED_FK</t>
+  </si>
+  <si>
+    <t>"APP"."CHILD"/FK_CHILD_PARENT</t>
+  </si>
+  <si>
+    <t>Omitted outgoing FK to "SHARED"."PARENT" because the parent table is not explicitly selected.</t>
   </si>
 </sst>
 </file>
@@ -845,7 +824,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="2">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -901,7 +880,7 @@
         <v>15</v>
       </c>
       <c r="B10" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -925,7 +904,7 @@
         <v>18</v>
       </c>
       <c r="B13" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -937,7 +916,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="12" customWidth="1"/>
@@ -1008,39 +987,9 @@
         <v>2</v>
       </c>
       <c r="I2" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J2" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H3" s="2">
-        <v>2</v>
-      </c>
-      <c r="I3" s="2">
-        <v>2</v>
-      </c>
-      <c r="J3" s="2">
         <v>1</v>
       </c>
     </row>
@@ -1053,7 +1002,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:U5"/>
+  <dimension ref="A1:U3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -1075,67 +1024,67 @@
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>22</v>
       </c>
       <c r="G1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="O1" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="O1" s="5" t="s">
+      <c r="R1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="T1" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>54</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="T1" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1152,14 +1101,14 @@
         <v>1</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G2" s="2"/>
       <c r="H2" s="3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="I2" s="3">
         <v>22</v>
@@ -1175,17 +1124,17 @@
         <v>0</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="O2" s="2"/>
       <c r="P2" s="3" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="S2" s="2"/>
       <c r="T2" s="2"/>
@@ -1205,12 +1154,12 @@
         <v>2</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
       <c r="H3" s="2" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="I3" s="2">
         <v>22</v>
@@ -1226,123 +1175,21 @@
         <v>0</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="O3" s="2"/>
       <c r="P3" s="2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="S3" s="2"/>
       <c r="T3" s="2"/>
       <c r="U3" s="2"/>
-    </row>
-    <row r="4" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="D4" s="3">
-        <v>1</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="I4" s="3">
-        <v>22</v>
-      </c>
-      <c r="J4" s="3">
-        <v>0</v>
-      </c>
-      <c r="K4" s="2"/>
-      <c r="L4" s="3">
-        <v>10</v>
-      </c>
-      <c r="M4" s="3">
-        <v>0</v>
-      </c>
-      <c r="N4" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="O4" s="2"/>
-      <c r="P4" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="Q4" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="R4" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="S4" s="2"/>
-      <c r="T4" s="2"/>
-      <c r="U4" s="2"/>
-    </row>
-    <row r="5" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D5" s="2">
-        <v>2</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="I5" s="2">
-        <v>22</v>
-      </c>
-      <c r="J5" s="2">
-        <v>0</v>
-      </c>
-      <c r="K5" s="2"/>
-      <c r="L5" s="2">
-        <v>10</v>
-      </c>
-      <c r="M5" s="2">
-        <v>0</v>
-      </c>
-      <c r="N5" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="O5" s="2"/>
-      <c r="P5" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="Q5" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="R5" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="S5" s="2"/>
-      <c r="T5" s="2"/>
-      <c r="U5" s="2"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:U1"/>
@@ -1353,7 +1200,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:T9"/>
+  <dimension ref="A1:T3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -1377,64 +1224,64 @@
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="L1" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="O1" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>77</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="2" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1445,52 +1292,46 @@
         <v>30</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="F2" s="3">
         <v>1</v>
       </c>
       <c r="G2" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="R2" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="H2" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="K2" s="3" t="s">
+      <c r="S2" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="L2" s="2"/>
-      <c r="M2" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="N2" s="2"/>
-      <c r="O2" s="2"/>
-      <c r="P2" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="Q2" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="R2" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="S2" s="3" t="s">
-        <v>61</v>
-      </c>
       <c r="T2" s="3" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1501,364 +1342,46 @@
         <v>30</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="F3" s="2">
         <v>2</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>62</v>
-      </c>
+        <v>59</v>
+      </c>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
       <c r="L3" s="2"/>
-      <c r="M3" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="N3" s="2"/>
-      <c r="O3" s="2"/>
+      <c r="M3" s="2"/>
+      <c r="N3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>78</v>
+      </c>
       <c r="P3" s="2" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="S3" s="2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="T3" s="2" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="4" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="F4" s="3">
-        <v>1</v>
-      </c>
-      <c r="G4" s="3" t="s">
         <v>58</v>
-      </c>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
-      <c r="M4" s="2"/>
-      <c r="N4" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="O4" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="P4" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="Q4" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="R4" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="S4" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="T4" s="3" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="5" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="F5" s="2">
-        <v>2</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
-      <c r="L5" s="2"/>
-      <c r="M5" s="2"/>
-      <c r="N5" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="O5" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="P5" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="Q5" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="R5" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="S5" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="T5" s="2" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="6" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="F6" s="3">
-        <v>1</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="I6" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="J6" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="K6" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="L6" s="2"/>
-      <c r="M6" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="N6" s="2"/>
-      <c r="O6" s="2"/>
-      <c r="P6" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="Q6" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="R6" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="S6" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="T6" s="3" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="7" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="F7" s="2">
-        <v>2</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="J7" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="K7" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="L7" s="2"/>
-      <c r="M7" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="N7" s="2"/>
-      <c r="O7" s="2"/>
-      <c r="P7" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="Q7" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="R7" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="S7" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="T7" s="2" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="8" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="F8" s="3">
-        <v>1</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
-      <c r="L8" s="2"/>
-      <c r="M8" s="2"/>
-      <c r="N8" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="O8" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="P8" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="Q8" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="R8" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="S8" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="T8" s="3" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="9" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="F9" s="2">
-        <v>2</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
-      <c r="L9" s="2"/>
-      <c r="M9" s="2"/>
-      <c r="N9" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="O9" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="P9" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="Q9" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="R9" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="S9" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="T9" s="2" t="s">
-        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -1870,7 +1393,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -1886,46 +1409,46 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="M1" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="N1" s="1" t="s">
         <v>92</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="M1" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="2" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1939,22 +1462,22 @@
         <v>29</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="J2" s="3" t="s">
         <v>34</v>
@@ -1963,11 +1486,11 @@
         <v>1</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="M2" s="2"/>
       <c r="N2" s="3" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1981,22 +1504,22 @@
         <v>29</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>34</v>
@@ -2005,95 +1528,11 @@
         <v>2</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="M3" s="2"/>
       <c r="N3" s="2" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="K4" s="3">
-        <v>1</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="M4" s="2"/>
-      <c r="N4" s="3" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="K5" s="2">
-        <v>2</v>
-      </c>
-      <c r="L5" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="M5" s="2"/>
-      <c r="N5" s="2" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -2122,43 +1561,43 @@
         <v>19</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>108</v>
+        <v>97</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>111</v>
+        <v>100</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="O1" s="5" t="s">
         <v>25</v>
@@ -2185,28 +1624,28 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>118</v>
-      </c>
       <c r="D1" s="1" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>121</v>
+        <v>110</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>122</v>
+        <v>111</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>123</v>
+        <v>112</v>
       </c>
     </row>
   </sheetData>
@@ -2230,22 +1669,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>124</v>
+        <v>113</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>125</v>
+        <v>114</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>126</v>
+        <v>115</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>123</v>
+        <v>112</v>
       </c>
     </row>
   </sheetData>
@@ -2257,7 +1696,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="12" customWidth="1"/>
@@ -2266,16 +1705,30 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>128</v>
+        <v>117</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>129</v>
+        <v>118</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>130</v>
+        <v>119</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>131</v>
+        <v>120</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>124</v>
       </c>
     </row>
   </sheetData>

</xml_diff>